<commit_message>
A* E2nK2G V2 Benchmark
</commit_message>
<xml_diff>
--- a/Algorithm Comparison.xlsx
+++ b/Algorithm Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alota\Desktop\Projects\Games\Project - Know the Space - A Dungeon's Puzzles I\Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DBA1471-2A8F-44C8-953E-DBAA19BE15BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B49ACD9-F858-4C99-88EF-117C2F3A7991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{477AD171-825F-4620-9280-6E07D4DDEAA7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="28">
   <si>
     <t>BFS</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>A* E2nK2G</t>
+  </si>
+  <si>
+    <t>A* E2nK2G V2</t>
   </si>
 </sst>
 </file>
@@ -370,7 +373,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -477,16 +480,10 @@
     <xf numFmtId="3" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -824,14 +821,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BCDCA76-CDD9-4BF0-BA41-307CB0FEB465}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
     <col min="2" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -871,11 +868,14 @@
       <c r="M1" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="27" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -915,15 +915,18 @@
       <c r="M2" s="28">
         <v>3</v>
       </c>
-      <c r="N2" s="6">
-        <v>3</v>
-      </c>
-      <c r="P2" s="35" t="s">
+      <c r="N2" s="28">
+        <v>3</v>
+      </c>
+      <c r="O2" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R2" s="35"/>
+    </row>
+    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -963,13 +966,16 @@
       <c r="M3" s="28">
         <v>5</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="28">
         <v>5</v>
       </c>
-      <c r="P3" s="35"/>
+      <c r="O3" s="6">
+        <v>5</v>
+      </c>
       <c r="Q3" s="35"/>
-    </row>
-    <row r="4" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R3" s="35"/>
+    </row>
+    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1009,11 +1015,14 @@
       <c r="M4" s="30">
         <v>1147</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="36">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="6">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1053,11 +1062,14 @@
       <c r="M5" s="30">
         <v>27705</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="36">
         <v>17982</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="6">
+        <v>17043</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -1097,11 +1109,14 @@
       <c r="M6" s="30">
         <v>429354</v>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="36">
         <v>116526</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O6" s="6">
+        <v>109399</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1141,11 +1156,14 @@
       <c r="M7" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="28">
         <v>99630</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O7" s="6">
+        <v>99630</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1185,11 +1203,14 @@
       <c r="M8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="28">
         <v>597633</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="6">
+        <v>558677</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1229,13 +1250,16 @@
       <c r="M9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="O9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="Q2:R3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1245,14 +1269,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{012AED55-E3FD-4933-A23F-5C3FD1988C65}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
     <col min="2" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
@@ -1292,11 +1316,14 @@
       <c r="M1" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="36" t="s">
+      <c r="N1" s="27" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -1336,15 +1363,18 @@
       <c r="M2" s="28">
         <v>3</v>
       </c>
-      <c r="N2" s="37">
-        <v>3</v>
-      </c>
-      <c r="P2" s="35" t="s">
+      <c r="N2" s="28">
+        <v>3</v>
+      </c>
+      <c r="O2" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R2" s="35"/>
+    </row>
+    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -1384,13 +1414,16 @@
       <c r="M3" s="28">
         <v>6</v>
       </c>
-      <c r="N3" s="37">
+      <c r="N3" s="28">
         <v>6</v>
       </c>
-      <c r="P3" s="35"/>
+      <c r="O3" s="6">
+        <v>6</v>
+      </c>
       <c r="Q3" s="35"/>
-    </row>
-    <row r="4" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R3" s="35"/>
+    </row>
+    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1430,11 +1463,14 @@
       <c r="M4" s="30">
         <v>2188</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="36">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="6">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1474,11 +1510,14 @@
       <c r="M5" s="30">
         <v>37031</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="36">
         <v>24979</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="6">
+        <v>23762</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -1518,11 +1557,14 @@
       <c r="M6" s="30">
         <v>572347</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="36">
         <v>142049</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O6" s="6">
+        <v>132691</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1562,11 +1604,14 @@
       <c r="M7" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N7" s="37">
+      <c r="N7" s="28">
         <v>132785</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O7" s="6">
+        <v>132785</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1606,11 +1651,14 @@
       <c r="M8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="37">
+      <c r="N8" s="28">
         <v>661807</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="6">
+        <v>618415</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1650,13 +1698,16 @@
       <c r="M9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="38" t="s">
+      <c r="N9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="O9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="Q2:R3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1665,14 +1716,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E30DF6C7-3687-40F8-8C26-44B4D757B9E6}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="17"/>
     <col min="2" max="16384" width="14.21875" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="17" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="17" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>18</v>
       </c>
@@ -1712,11 +1763,14 @@
       <c r="M1" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="31" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
@@ -1756,15 +1810,18 @@
       <c r="M2" s="32">
         <v>1E-3</v>
       </c>
-      <c r="N2" s="20">
+      <c r="N2" s="32">
         <v>2E-3</v>
       </c>
-      <c r="P2" s="35" t="s">
+      <c r="O2" s="20">
+        <v>1E-3</v>
+      </c>
+      <c r="Q2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R2" s="35"/>
+    </row>
+    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
         <v>10</v>
       </c>
@@ -1804,13 +1861,16 @@
       <c r="M3" s="32">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="N3" s="20">
+      <c r="N3" s="32">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="P3" s="35"/>
+      <c r="O3" s="20">
+        <v>2E-3</v>
+      </c>
       <c r="Q3" s="35"/>
-    </row>
-    <row r="4" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R3" s="35"/>
+    </row>
+    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>11</v>
       </c>
@@ -1850,11 +1910,14 @@
       <c r="M4" s="34">
         <v>1.9670000000000001</v>
       </c>
-      <c r="N4" s="39">
+      <c r="N4" s="37">
         <v>2.9000000000000001E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="20">
+        <v>2.3E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>12</v>
       </c>
@@ -1894,11 +1957,14 @@
       <c r="M5" s="34">
         <v>61.040999999999997</v>
       </c>
-      <c r="N5" s="39">
+      <c r="N5" s="37">
         <v>38.517000000000003</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="20">
+        <v>32.631999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
         <v>13</v>
       </c>
@@ -1938,11 +2004,14 @@
       <c r="M6" s="34">
         <v>1437.423</v>
       </c>
-      <c r="N6" s="39">
+      <c r="N6" s="37">
         <v>309.14299999999997</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O6" s="20">
+        <v>259.50200000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
         <v>14</v>
       </c>
@@ -1982,11 +2051,14 @@
       <c r="M7" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="N7" s="20">
+      <c r="N7" s="32">
         <v>260.83699999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O7" s="20">
+        <v>224.27500000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
         <v>15</v>
       </c>
@@ -2026,11 +2098,14 @@
       <c r="M8" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="20">
+      <c r="N8" s="32">
         <v>2227.92</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="20">
+        <v>1742.0229999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
         <v>16</v>
       </c>
@@ -2070,13 +2145,16 @@
       <c r="M9" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="26" t="s">
+      <c r="N9" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="O9" s="26" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="Q2:R3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2085,14 +2163,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72C608C-3462-4F97-9DBB-2A960F7121A5}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
     <col min="2" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>17</v>
       </c>
@@ -2132,11 +2210,14 @@
       <c r="M1" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="31" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -2176,15 +2257,18 @@
       <c r="M2" s="28">
         <v>2</v>
       </c>
-      <c r="N2" s="6">
+      <c r="N2" s="28">
         <v>2</v>
       </c>
-      <c r="P2" s="35" t="s">
+      <c r="O2" s="6">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="35"/>
-    </row>
-    <row r="3" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R2" s="35"/>
+    </row>
+    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -2224,13 +2308,16 @@
       <c r="M3" s="28">
         <v>4</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="28">
         <v>4</v>
       </c>
-      <c r="P3" s="35"/>
+      <c r="O3" s="6">
+        <v>4</v>
+      </c>
       <c r="Q3" s="35"/>
-    </row>
-    <row r="4" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R3" s="35"/>
+    </row>
+    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -2270,11 +2357,14 @@
       <c r="M4" s="30">
         <v>9</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="36">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -2314,11 +2404,14 @@
       <c r="M5" s="30">
         <v>25</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="36">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -2358,11 +2451,14 @@
       <c r="M6" s="30">
         <v>56</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="36">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O6" s="6">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -2402,11 +2498,14 @@
       <c r="M7" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="28">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O7" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -2446,11 +2545,14 @@
       <c r="M8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="28">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="6">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -2490,13 +2592,16 @@
       <c r="M9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="O9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="Q2:R3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
A* E2nK2G V2 + Connected Goal (CG) Benchmark
</commit_message>
<xml_diff>
--- a/Algorithm Comparison.xlsx
+++ b/Algorithm Comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alota\Desktop\Projects\Games\Project - Know the Space - A Dungeon's Puzzles I\Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B49ACD9-F858-4C99-88EF-117C2F3A7991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2561400A-83F3-4FA6-841D-07B978E33A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{477AD171-825F-4620-9280-6E07D4DDEAA7}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="29">
   <si>
     <t>BFS</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>A* E2nK2G V2</t>
+  </si>
+  <si>
+    <t>A* E2nK2G V2 + CG</t>
   </si>
 </sst>
 </file>
@@ -373,7 +376,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -479,12 +482,6 @@
     </xf>
     <xf numFmtId="3" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -821,14 +818,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BCDCA76-CDD9-4BF0-BA41-307CB0FEB465}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
-    <col min="2" max="16384" width="14.21875" style="7"/>
+    <col min="2" max="15" width="14.21875" style="7"/>
+    <col min="16" max="16" width="18.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -871,11 +870,14 @@
       <c r="N1" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="27" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -918,15 +920,18 @@
       <c r="N2" s="28">
         <v>3</v>
       </c>
-      <c r="O2" s="6">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="35" t="s">
+      <c r="O2" s="28">
+        <v>3</v>
+      </c>
+      <c r="P2" s="6">
+        <v>3</v>
+      </c>
+      <c r="R2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="35"/>
-    </row>
-    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S2" s="35"/>
+    </row>
+    <row r="3" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -969,13 +974,16 @@
       <c r="N3" s="28">
         <v>5</v>
       </c>
-      <c r="O3" s="6">
+      <c r="O3" s="28">
         <v>5</v>
       </c>
-      <c r="Q3" s="35"/>
+      <c r="P3" s="6">
+        <v>5</v>
+      </c>
       <c r="R3" s="35"/>
-    </row>
-    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S3" s="35"/>
+    </row>
+    <row r="4" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1015,14 +1023,17 @@
       <c r="M4" s="30">
         <v>1147</v>
       </c>
-      <c r="N4" s="36">
+      <c r="N4" s="28">
         <v>18</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="28">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="6">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1062,14 +1073,17 @@
       <c r="M5" s="30">
         <v>27705</v>
       </c>
-      <c r="N5" s="36">
+      <c r="N5" s="28">
         <v>17982</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="28">
         <v>17043</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P5" s="6">
+        <v>8453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -1109,14 +1123,17 @@
       <c r="M6" s="30">
         <v>429354</v>
       </c>
-      <c r="N6" s="36">
+      <c r="N6" s="28">
         <v>116526</v>
       </c>
-      <c r="O6" s="6">
+      <c r="O6" s="28">
         <v>109399</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P6" s="6">
+        <v>76100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1159,11 +1176,14 @@
       <c r="N7" s="28">
         <v>99630</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="28">
         <v>99630</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="6">
+        <v>25532</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1206,11 +1226,14 @@
       <c r="N8" s="28">
         <v>597633</v>
       </c>
-      <c r="O8" s="6">
+      <c r="O8" s="28">
         <v>558677</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1253,13 +1276,16 @@
       <c r="N9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:R3"/>
+    <mergeCell ref="R2:S3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1269,14 +1295,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{012AED55-E3FD-4933-A23F-5C3FD1988C65}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
-    <col min="2" max="16384" width="14.21875" style="7"/>
+    <col min="2" max="15" width="14.21875" style="7"/>
+    <col min="16" max="16" width="18.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
@@ -1319,11 +1347,14 @@
       <c r="N1" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="27" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -1366,15 +1397,18 @@
       <c r="N2" s="28">
         <v>3</v>
       </c>
-      <c r="O2" s="6">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="35" t="s">
+      <c r="O2" s="28">
+        <v>3</v>
+      </c>
+      <c r="P2" s="6">
+        <v>3</v>
+      </c>
+      <c r="R2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="35"/>
-    </row>
-    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S2" s="35"/>
+    </row>
+    <row r="3" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -1417,13 +1451,16 @@
       <c r="N3" s="28">
         <v>6</v>
       </c>
-      <c r="O3" s="6">
+      <c r="O3" s="28">
         <v>6</v>
       </c>
-      <c r="Q3" s="35"/>
+      <c r="P3" s="6">
+        <v>6</v>
+      </c>
       <c r="R3" s="35"/>
-    </row>
-    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S3" s="35"/>
+    </row>
+    <row r="4" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -1463,14 +1500,17 @@
       <c r="M4" s="30">
         <v>2188</v>
       </c>
-      <c r="N4" s="36">
+      <c r="N4" s="28">
         <v>45</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="28">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="6">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1510,14 +1550,17 @@
       <c r="M5" s="30">
         <v>37031</v>
       </c>
-      <c r="N5" s="36">
+      <c r="N5" s="28">
         <v>24979</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="28">
         <v>23762</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P5" s="6">
+        <v>12073</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -1557,14 +1600,17 @@
       <c r="M6" s="30">
         <v>572347</v>
       </c>
-      <c r="N6" s="36">
+      <c r="N6" s="28">
         <v>142049</v>
       </c>
-      <c r="O6" s="6">
+      <c r="O6" s="28">
         <v>132691</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P6" s="6">
+        <v>94228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1607,11 +1653,14 @@
       <c r="N7" s="28">
         <v>132785</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="28">
         <v>132785</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="6">
+        <v>38108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -1654,11 +1703,14 @@
       <c r="N8" s="28">
         <v>661807</v>
       </c>
-      <c r="O8" s="6">
+      <c r="O8" s="28">
         <v>618415</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -1701,13 +1753,16 @@
       <c r="N9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:R3"/>
+    <mergeCell ref="R2:S3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1716,14 +1771,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E30DF6C7-3687-40F8-8C26-44B4D757B9E6}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="17"/>
-    <col min="2" max="16384" width="14.21875" style="21"/>
+    <col min="2" max="15" width="14.21875" style="21"/>
+    <col min="16" max="16" width="18.88671875" style="21" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="14.21875" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="17" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="17" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>18</v>
       </c>
@@ -1766,11 +1823,14 @@
       <c r="N1" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="31" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
@@ -1813,15 +1873,18 @@
       <c r="N2" s="32">
         <v>2E-3</v>
       </c>
-      <c r="O2" s="20">
+      <c r="O2" s="32">
         <v>1E-3</v>
       </c>
-      <c r="Q2" s="35" t="s">
+      <c r="P2" s="20">
+        <v>2E-3</v>
+      </c>
+      <c r="R2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="35"/>
-    </row>
-    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S2" s="35"/>
+    </row>
+    <row r="3" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
         <v>10</v>
       </c>
@@ -1864,13 +1927,16 @@
       <c r="N3" s="32">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="O3" s="20">
+      <c r="O3" s="32">
         <v>2E-3</v>
       </c>
-      <c r="Q3" s="35"/>
+      <c r="P3" s="20">
+        <v>5.0000000000000001E-3</v>
+      </c>
       <c r="R3" s="35"/>
-    </row>
-    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S3" s="35"/>
+    </row>
+    <row r="4" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>11</v>
       </c>
@@ -1910,14 +1976,17 @@
       <c r="M4" s="34">
         <v>1.9670000000000001</v>
       </c>
-      <c r="N4" s="37">
+      <c r="N4" s="32">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="O4" s="20">
+      <c r="O4" s="32">
         <v>2.3E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="20">
+        <v>3.3000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
         <v>12</v>
       </c>
@@ -1957,14 +2026,17 @@
       <c r="M5" s="34">
         <v>61.040999999999997</v>
       </c>
-      <c r="N5" s="37">
+      <c r="N5" s="32">
         <v>38.517000000000003</v>
       </c>
-      <c r="O5" s="20">
+      <c r="O5" s="32">
         <v>32.631999999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P5" s="20">
+        <v>29.753</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
         <v>13</v>
       </c>
@@ -2004,14 +2076,17 @@
       <c r="M6" s="34">
         <v>1437.423</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="32">
         <v>309.14299999999997</v>
       </c>
-      <c r="O6" s="20">
+      <c r="O6" s="32">
         <v>259.50200000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P6" s="20">
+        <v>2802.1010000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
         <v>14</v>
       </c>
@@ -2054,11 +2129,14 @@
       <c r="N7" s="32">
         <v>260.83699999999999</v>
       </c>
-      <c r="O7" s="20">
+      <c r="O7" s="32">
         <v>224.27500000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="20">
+        <v>522.62300000000005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
         <v>15</v>
       </c>
@@ -2101,11 +2179,14 @@
       <c r="N8" s="32">
         <v>2227.92</v>
       </c>
-      <c r="O8" s="20">
+      <c r="O8" s="32">
         <v>1742.0229999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
         <v>16</v>
       </c>
@@ -2148,13 +2229,16 @@
       <c r="N9" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="O9" s="26" t="s">
+      <c r="O9" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="26" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:R3"/>
+    <mergeCell ref="R2:S3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2163,14 +2247,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72C608C-3462-4F97-9DBB-2A960F7121A5}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultColWidth="14.21875" defaultRowHeight="38.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" style="3"/>
-    <col min="2" max="16384" width="14.21875" style="7"/>
+    <col min="2" max="15" width="14.21875" style="7"/>
+    <col min="16" max="16" width="18.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="14.21875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="3" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>17</v>
       </c>
@@ -2213,11 +2299,14 @@
       <c r="N1" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="31" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P1" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -2260,15 +2349,18 @@
       <c r="N2" s="28">
         <v>2</v>
       </c>
-      <c r="O2" s="6">
+      <c r="O2" s="28">
         <v>2</v>
       </c>
-      <c r="Q2" s="35" t="s">
+      <c r="P2" s="6">
+        <v>2</v>
+      </c>
+      <c r="R2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="35"/>
-    </row>
-    <row r="3" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S2" s="35"/>
+    </row>
+    <row r="3" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -2311,13 +2403,16 @@
       <c r="N3" s="28">
         <v>4</v>
       </c>
-      <c r="O3" s="6">
+      <c r="O3" s="28">
         <v>4</v>
       </c>
-      <c r="Q3" s="35"/>
+      <c r="P3" s="6">
+        <v>4</v>
+      </c>
       <c r="R3" s="35"/>
-    </row>
-    <row r="4" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S3" s="35"/>
+    </row>
+    <row r="4" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
@@ -2357,14 +2452,17 @@
       <c r="M4" s="30">
         <v>9</v>
       </c>
-      <c r="N4" s="36">
+      <c r="N4" s="28">
         <v>8</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="28">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -2404,14 +2502,17 @@
       <c r="M5" s="30">
         <v>25</v>
       </c>
-      <c r="N5" s="36">
+      <c r="N5" s="28">
         <v>24</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="28">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P5" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -2451,14 +2552,17 @@
       <c r="M6" s="30">
         <v>56</v>
       </c>
-      <c r="N6" s="36">
+      <c r="N6" s="28">
         <v>47</v>
       </c>
-      <c r="O6" s="6">
+      <c r="O6" s="28">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P6" s="6">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -2501,11 +2605,14 @@
       <c r="N7" s="28">
         <v>30</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="28">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
@@ -2548,11 +2655,14 @@
       <c r="N8" s="28">
         <v>45</v>
       </c>
-      <c r="O8" s="6">
+      <c r="O8" s="28">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>16</v>
       </c>
@@ -2595,13 +2705,16 @@
       <c r="N9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="P9" s="12" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q2:R3"/>
+    <mergeCell ref="R2:S3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>